<commit_message>
Auto-refresh fixtures from Dribl (2026-09-29)
</commit_message>
<xml_diff>
--- a/Manningham_fixtures_and_overlaps.xlsx
+++ b/Manningham_fixtures_and_overlaps.xlsx
@@ -596,7 +596,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Source: fv.dribl.com, 2026 season, generated 28 Sep 2026</t>
+          <t>Source: fv.dribl.com, 2026 season, generated 29 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -27314,7 +27314,7 @@
       </c>
       <c r="L353" s="12" t="inlineStr">
         <is>
-          <t>Darebin Womens SC U13</t>
+          <t>Darebin Falcons Womens SC U13</t>
         </is>
       </c>
       <c r="M353" s="12" t="inlineStr">
@@ -27391,7 +27391,7 @@
       </c>
       <c r="L354" s="10" t="inlineStr">
         <is>
-          <t>Darebin Womens SC U15</t>
+          <t>Darebin Falcons Womens SC U15</t>
         </is>
       </c>
       <c r="M354" s="10" t="inlineStr">
@@ -27468,7 +27468,7 @@
       </c>
       <c r="L355" s="12" t="inlineStr">
         <is>
-          <t>Darebin Womens SC U17</t>
+          <t>Darebin Falcons Womens SC U17</t>
         </is>
       </c>
       <c r="M355" s="12" t="inlineStr">
@@ -44462,7 +44462,7 @@
       </c>
       <c r="L577" s="12" t="inlineStr">
         <is>
-          <t>Darebin Womens SC U09 MiniRoos - Wallabies Female Darebin Falcons Red</t>
+          <t>Darebin Falcons Womens SC U09 MiniRoos - Wallabies Female Darebin Falcons Red</t>
         </is>
       </c>
       <c r="M577" s="12" t="inlineStr">

</xml_diff>